<commit_message>
major debugging; rewriting of PV Earnings report template; etc.
</commit_message>
<xml_diff>
--- a/EconAutomation/src/supporting_docs/econ_wb_templates/Case_Variables.xlsx
+++ b/EconAutomation/src/supporting_docs/econ_wb_templates/Case_Variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricBussey\GitHub\EconAutomation-REP\EconAutomation\src\supporting_docs\econ_wb_templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmacbook/Documents/GitHub/EconAutomation-REP/EconAutomation/src/supporting_docs/econ_wb_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C378A4DD-2272-474A-814E-35A4C5BAA1C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88BB1DF8-7904-9646-A5B6-0A4CFFB99F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{765FF91D-C91B-E74A-AE6E-CE36BB29D05E}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="32000" windowHeight="20080" xr2:uid="{765FF91D-C91B-E74A-AE6E-CE36BB29D05E}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORT_OUTPUTS" sheetId="3" r:id="rId1"/>
@@ -477,7 +477,7 @@
       <name val="Aptos Display"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,12 +504,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -527,7 +521,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -536,34 +530,21 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
       </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
+      <left style="medium">
         <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
       </left>
       <right style="thin">
         <color theme="0" tint="-0.14999847407452621"/>
@@ -580,6 +561,77 @@
       <left style="thin">
         <color theme="0" tint="-0.14999847407452621"/>
       </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color theme="0" tint="-0.14999847407452621"/>
       </right>
@@ -593,10 +645,10 @@
       <left style="thin">
         <color theme="0" tint="-0.14999847407452621"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </top>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color theme="0" tint="-0.14999847407452621"/>
       </bottom>
@@ -613,7 +665,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -710,118 +762,97 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="17" fillId="2" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="17" fillId="0" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="18" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="18" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Currency 2" xfId="3" xr:uid="{094F03E6-2C7C-534A-9A60-E576CB1D5C44}"/>
@@ -831,7 +862,388 @@
     <cellStyle name="Normal 2" xfId="2" xr:uid="{6F2027E1-5DA8-B64C-9928-C7D64A51A230}"/>
     <cellStyle name="Percent 2" xfId="4" xr:uid="{F9E35F16-9AB0-2F47-9A1E-E8B3AF0707E3}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top style="thin">
+          <color theme="0"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right style="thin">
+          <color theme="0" tint="-0.14996795556505021"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top style="thin">
+          <color theme="0"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top style="thin">
+          <color theme="0"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top style="thin">
+          <color theme="0"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top style="thin">
+          <color theme="0"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1165,1150 +1577,1148 @@
     <tabColor theme="6" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:M230"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="37.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="35" style="1" customWidth="1"/>
+    <col min="2" max="2" width="31.83203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="18.5" style="1" customWidth="1"/>
     <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
     <col min="5" max="6" width="9" style="1"/>
-    <col min="7" max="7" width="12.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="15" style="1" customWidth="1"/>
-    <col min="9" max="9" width="18.125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.1640625" style="1" customWidth="1"/>
     <col min="10" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:3" ht="25" x14ac:dyDescent="0.15">
+      <c r="A1" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="70"/>
-    </row>
-    <row r="2" spans="1:5" ht="21" x14ac:dyDescent="0.2">
-      <c r="A2" s="69" t="s">
+      <c r="B1" s="55"/>
+      <c r="C1" s="36"/>
+    </row>
+    <row r="2" spans="1:3" ht="20" x14ac:dyDescent="0.15">
+      <c r="A2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="69"/>
+      <c r="B2" s="54"/>
       <c r="C2" s="31"/>
     </row>
-    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="40" t="s">
+    <row r="3" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A3" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="41"/>
+      <c r="B3" s="53"/>
       <c r="C3" s="32"/>
     </row>
-    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="42" t="s">
+    <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A4" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="43"/>
+      <c r="B4" s="38"/>
       <c r="C4" s="22"/>
     </row>
-    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="40" t="s">
+    <row r="5" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A5" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="44"/>
+      <c r="B5" s="38"/>
       <c r="C5" s="22"/>
     </row>
-    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="42" t="s">
+    <row r="6" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A6" s="58" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="43"/>
+      <c r="B6" s="38"/>
       <c r="C6" s="22"/>
     </row>
-    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="40" t="s">
+    <row r="7" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A7" s="58" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="45"/>
+      <c r="B7" s="38"/>
       <c r="C7" s="12"/>
     </row>
-    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="42" t="s">
+    <row r="8" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A8" s="58" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="46"/>
+      <c r="B8" s="38"/>
       <c r="C8" s="12"/>
-      <c r="E8" s="71"/>
-    </row>
-    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A9" s="40" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A9" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="47"/>
+      <c r="B9" s="38"/>
       <c r="C9" s="12"/>
-      <c r="E9" s="71"/>
-    </row>
-    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A10" s="42" t="s">
+    </row>
+    <row r="10" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A10" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="48"/>
+      <c r="B10" s="38"/>
       <c r="C10" s="17"/>
     </row>
-    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A11" s="40" t="s">
+    <row r="11" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A11" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="72"/>
-      <c r="C11" s="73"/>
-    </row>
-    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A12" s="42" t="s">
+      <c r="B11" s="38"/>
+      <c r="C11" s="17"/>
+    </row>
+    <row r="12" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A12" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="73"/>
-    </row>
-    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A13" s="40" t="s">
+      <c r="B12" s="38"/>
+      <c r="C12" s="17"/>
+    </row>
+    <row r="13" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A13" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="50"/>
+      <c r="B13" s="38"/>
       <c r="C13" s="17"/>
     </row>
-    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A14" s="42" t="s">
+    <row r="14" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A14" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="48"/>
+      <c r="B14" s="38"/>
       <c r="C14" s="17"/>
     </row>
-    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A15" s="40" t="s">
+    <row r="15" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A15" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="51"/>
+      <c r="B15" s="39"/>
       <c r="C15" s="17"/>
     </row>
-    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A16" s="42" t="s">
+    <row r="16" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A16" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="52"/>
+      <c r="B16" s="39"/>
       <c r="C16" s="17"/>
     </row>
-    <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A17" s="40" t="s">
+    <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A17" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="B17" s="53"/>
+      <c r="B17" s="39"/>
       <c r="C17" s="17"/>
     </row>
-    <row r="18" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A18" s="42" t="s">
+    <row r="18" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A18" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="52"/>
+      <c r="B18" s="39"/>
       <c r="C18" s="17"/>
     </row>
-    <row r="19" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A19" s="40" t="s">
+    <row r="19" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A19" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="53"/>
+      <c r="B19" s="39"/>
       <c r="C19" s="17"/>
     </row>
-    <row r="20" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A20" s="42" t="s">
+    <row r="20" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A20" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="52"/>
+      <c r="B20" s="39"/>
       <c r="C20" s="17"/>
     </row>
-    <row r="21" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A21" s="40" t="s">
+    <row r="21" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A21" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="45"/>
+      <c r="B21" s="38"/>
       <c r="C21" s="26"/>
     </row>
-    <row r="22" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A22" s="42" t="s">
+    <row r="22" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A22" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="54"/>
+      <c r="B22" s="38"/>
       <c r="C22" s="26"/>
     </row>
-    <row r="23" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A23" s="40" t="s">
+    <row r="23" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A23" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="51"/>
+      <c r="B23" s="39"/>
       <c r="C23" s="26"/>
     </row>
-    <row r="24" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A24" s="42" t="s">
+    <row r="24" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A24" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="55"/>
+      <c r="B24" s="39"/>
       <c r="C24" s="26"/>
     </row>
-    <row r="25" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A25" s="40" t="s">
+    <row r="25" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A25" s="58" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="51"/>
+      <c r="B25" s="39"/>
       <c r="C25" s="26"/>
     </row>
-    <row r="26" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A26" s="42" t="s">
+    <row r="26" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A26" s="58" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="55"/>
+      <c r="B26" s="39"/>
       <c r="C26" s="26"/>
     </row>
-    <row r="27" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A27" s="40" t="s">
+    <row r="27" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A27" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="51"/>
+      <c r="B27" s="39"/>
       <c r="C27" s="26"/>
     </row>
-    <row r="28" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A28" s="42" t="s">
+    <row r="28" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A28" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="55"/>
+      <c r="B28" s="39"/>
       <c r="C28" s="26"/>
     </row>
-    <row r="29" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A29" s="40" t="s">
+    <row r="29" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A29" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="51"/>
+      <c r="B29" s="39"/>
       <c r="C29" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A30" s="42" t="s">
+    <row r="30" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A30" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="B30" s="55"/>
+      <c r="B30" s="39"/>
       <c r="C30" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A31" s="40" t="s">
+    <row r="31" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A31" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="51"/>
+      <c r="B31" s="39"/>
       <c r="C31" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A32" s="42" t="s">
+    <row r="32" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A32" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B32" s="55"/>
+      <c r="B32" s="39"/>
       <c r="C32" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A33" s="38" t="s">
+    <row r="33" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A33" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="51"/>
+      <c r="B33" s="39"/>
       <c r="C33" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A34" s="42" t="s">
+    <row r="34" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+      <c r="A34" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="56"/>
+      <c r="B34" s="40"/>
       <c r="C34" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35" s="38" t="s">
+    <row r="35" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A35" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="39"/>
+      <c r="B35" s="41"/>
       <c r="C35" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A36" s="42" t="s">
+    <row r="36" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A36" s="58" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="57"/>
+      <c r="B36" s="41"/>
       <c r="C36" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A37" s="38" t="s">
+    <row r="37" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A37" s="58" t="s">
         <v>69</v>
       </c>
-      <c r="B37" s="39"/>
+      <c r="B37" s="41"/>
       <c r="C37" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38" s="42" t="s">
+    <row r="38" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A38" s="58" t="s">
         <v>70</v>
       </c>
-      <c r="B38" s="57"/>
+      <c r="B38" s="41"/>
       <c r="C38" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39" s="38" t="s">
+    <row r="39" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A39" s="58" t="s">
         <v>71</v>
       </c>
-      <c r="B39" s="39"/>
+      <c r="B39" s="41"/>
       <c r="C39" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="42"/>
-      <c r="B40" s="57"/>
+    <row r="40" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A40" s="58"/>
+      <c r="B40" s="41"/>
       <c r="C40" s="14"/>
     </row>
-    <row r="41" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41" s="74"/>
-      <c r="B41" s="75"/>
+    <row r="41" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A41" s="59"/>
+      <c r="B41" s="51"/>
       <c r="C41" s="14"/>
     </row>
-    <row r="42" spans="1:3" ht="21" x14ac:dyDescent="0.2">
-      <c r="A42" s="67" t="s">
+    <row r="42" spans="1:3" ht="20" x14ac:dyDescent="0.15">
+      <c r="A42" s="52" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="67"/>
+      <c r="B42" s="52"/>
       <c r="C42" s="33"/>
     </row>
-    <row r="43" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A43" s="39" t="s">
+    <row r="43" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A43" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="B43" s="39"/>
-    </row>
-    <row r="44" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A44" s="57" t="s">
+      <c r="B43" s="49"/>
+    </row>
+    <row r="44" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A44" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="B44" s="57"/>
-    </row>
-    <row r="45" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A45" s="39" t="s">
+      <c r="B44" s="43"/>
+    </row>
+    <row r="45" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A45" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="B45" s="39"/>
-    </row>
-    <row r="46" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="57" t="s">
+      <c r="B45" s="42"/>
+    </row>
+    <row r="46" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A46" s="61" t="s">
         <v>74</v>
       </c>
-      <c r="B46" s="57"/>
-    </row>
-    <row r="47" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A47" s="75" t="s">
+      <c r="B46" s="43"/>
+    </row>
+    <row r="47" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A47" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="B47" s="75"/>
-    </row>
-    <row r="48" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A48" s="57" t="s">
+      <c r="B47" s="44"/>
+    </row>
+    <row r="48" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A48" s="61" t="s">
         <v>40</v>
       </c>
-      <c r="B48" s="57"/>
-    </row>
-    <row r="49" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49" s="75" t="s">
+      <c r="B48" s="43"/>
+    </row>
+    <row r="49" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A49" s="63" t="s">
         <v>75</v>
       </c>
-      <c r="B49" s="75"/>
-    </row>
-    <row r="50" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="57" t="s">
+      <c r="B49" s="44"/>
+    </row>
+    <row r="50" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A50" s="61" t="s">
         <v>76</v>
       </c>
-      <c r="B50" s="57"/>
-    </row>
-    <row r="51" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A51" s="75" t="s">
+      <c r="B50" s="43"/>
+    </row>
+    <row r="51" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A51" s="63" t="s">
         <v>61</v>
       </c>
-      <c r="B51" s="75"/>
+      <c r="B51" s="44"/>
       <c r="C51" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A52" s="57" t="s">
+    <row r="52" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A52" s="61" t="s">
         <v>62</v>
       </c>
-      <c r="B52" s="57"/>
+      <c r="B52" s="43"/>
       <c r="C52" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A53" s="75" t="s">
+    <row r="53" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A53" s="63" t="s">
         <v>63</v>
       </c>
-      <c r="B53" s="75"/>
+      <c r="B53" s="44"/>
       <c r="C53" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A54" s="57" t="s">
+    <row r="54" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A54" s="61" t="s">
         <v>64</v>
       </c>
-      <c r="B54" s="57"/>
+      <c r="B54" s="43"/>
       <c r="C54" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A55" s="75" t="s">
+    <row r="55" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A55" s="63" t="s">
         <v>65</v>
       </c>
-      <c r="B55" s="75"/>
+      <c r="B55" s="44"/>
       <c r="C55" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A56" s="57" t="s">
+    <row r="56" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A56" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="B56" s="57"/>
-    </row>
-    <row r="57" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A57" s="75" t="s">
+      <c r="B56" s="43"/>
+    </row>
+    <row r="57" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A57" s="63" t="s">
         <v>42</v>
       </c>
-      <c r="B57" s="75"/>
-    </row>
-    <row r="58" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A58" s="57" t="s">
+      <c r="B57" s="44"/>
+    </row>
+    <row r="58" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A58" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="B58" s="57"/>
-    </row>
-    <row r="59" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A59" s="75" t="s">
+      <c r="B58" s="43"/>
+    </row>
+    <row r="59" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A59" s="63" t="s">
         <v>44</v>
       </c>
-      <c r="B59" s="75"/>
-    </row>
-    <row r="60" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A60" s="57"/>
-      <c r="B60" s="57"/>
-    </row>
-    <row r="61" spans="1:3" ht="21" x14ac:dyDescent="0.35">
-      <c r="A61" s="68" t="s">
+      <c r="B59" s="44"/>
+    </row>
+    <row r="60" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A60" s="64"/>
+      <c r="B60" s="48"/>
+    </row>
+    <row r="61" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+      <c r="A61" s="50" t="s">
         <v>67</v>
       </c>
-      <c r="B61" s="68"/>
+      <c r="B61" s="50"/>
       <c r="C61" s="34"/>
     </row>
-    <row r="62" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A62" s="39" t="s">
+    <row r="62" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A62" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="B62" s="39"/>
-    </row>
-    <row r="63" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A63" s="57" t="s">
+      <c r="B62" s="49"/>
+    </row>
+    <row r="63" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A63" s="61" t="s">
         <v>12</v>
       </c>
-      <c r="B63" s="57"/>
-    </row>
-    <row r="64" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A64" s="39" t="s">
+      <c r="B63" s="43"/>
+    </row>
+    <row r="64" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A64" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="B64" s="39"/>
-    </row>
-    <row r="65" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A65" s="57" t="s">
+      <c r="B64" s="42"/>
+    </row>
+    <row r="65" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A65" s="61" t="s">
         <v>45</v>
       </c>
-      <c r="B65" s="57"/>
-    </row>
-    <row r="66" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A66" s="39" t="s">
+      <c r="B65" s="43"/>
+    </row>
+    <row r="66" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A66" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="B66" s="39"/>
-    </row>
-    <row r="67" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A67" s="57" t="s">
+      <c r="B66" s="42"/>
+    </row>
+    <row r="67" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A67" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="B67" s="57"/>
-    </row>
-    <row r="68" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A68" s="39" t="s">
+      <c r="B67" s="43"/>
+    </row>
+    <row r="68" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A68" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="B68" s="39"/>
-    </row>
-    <row r="69" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A69" s="57" t="s">
+      <c r="B68" s="42"/>
+    </row>
+    <row r="69" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A69" s="61" t="s">
         <v>14</v>
       </c>
-      <c r="B69" s="57"/>
-    </row>
-    <row r="70" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A70" s="39" t="s">
+      <c r="B69" s="43"/>
+    </row>
+    <row r="70" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A70" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="B70" s="39"/>
+      <c r="B70" s="42"/>
       <c r="M70" s="2"/>
     </row>
-    <row r="71" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A71" s="57" t="s">
+    <row r="71" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A71" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="B71" s="57"/>
+      <c r="B71" s="43"/>
       <c r="M71" s="2"/>
     </row>
-    <row r="72" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A72" s="39" t="s">
+    <row r="72" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A72" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="B72" s="39"/>
+      <c r="B72" s="42"/>
       <c r="M72" s="2"/>
     </row>
-    <row r="73" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A73" s="57" t="s">
+    <row r="73" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A73" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="B73" s="57"/>
+      <c r="B73" s="43"/>
       <c r="M73" s="2"/>
     </row>
-    <row r="74" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A74" s="39" t="s">
+    <row r="74" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A74" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="B74" s="39"/>
+      <c r="B74" s="42"/>
       <c r="M74" s="2"/>
     </row>
-    <row r="75" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A75" s="58" t="s">
+    <row r="75" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A75" s="61" t="s">
         <v>50</v>
       </c>
-      <c r="B75" s="57"/>
+      <c r="B75" s="43"/>
       <c r="M75" s="2"/>
     </row>
-    <row r="76" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A76" s="59" t="s">
+    <row r="76" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A76" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="B76" s="39"/>
+      <c r="B76" s="42"/>
       <c r="M76" s="2"/>
     </row>
-    <row r="77" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A77" s="58" t="s">
+    <row r="77" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A77" s="61" t="s">
         <v>52</v>
       </c>
-      <c r="B77" s="57"/>
+      <c r="B77" s="43"/>
       <c r="M77" s="2"/>
     </row>
-    <row r="78" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A78" s="59" t="s">
+    <row r="78" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A78" s="62" t="s">
         <v>53</v>
       </c>
-      <c r="B78" s="39"/>
+      <c r="B78" s="42"/>
       <c r="M78" s="2"/>
     </row>
-    <row r="79" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A79" s="57" t="s">
+    <row r="79" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A79" s="61" t="s">
         <v>54</v>
       </c>
-      <c r="B79" s="57"/>
+      <c r="B79" s="43"/>
       <c r="M79" s="2"/>
     </row>
-    <row r="80" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A80" s="39"/>
-      <c r="B80" s="39"/>
+    <row r="80" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A80" s="65"/>
+      <c r="B80" s="56"/>
       <c r="M80" s="2"/>
     </row>
-    <row r="81" spans="1:13" ht="21" x14ac:dyDescent="0.35">
-      <c r="A81" s="68" t="s">
+    <row r="81" spans="1:13" ht="20" x14ac:dyDescent="0.25">
+      <c r="A81" s="50" t="s">
         <v>77</v>
       </c>
-      <c r="B81" s="68"/>
+      <c r="B81" s="50"/>
       <c r="C81" s="34"/>
       <c r="M81" s="2"/>
     </row>
-    <row r="82" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A82" s="39"/>
-      <c r="B82" s="39"/>
+    <row r="82" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A82" s="60"/>
+      <c r="B82" s="49"/>
       <c r="M82" s="2"/>
     </row>
-    <row r="83" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A83" s="57"/>
-      <c r="B83" s="57"/>
+    <row r="83" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A83" s="61"/>
+      <c r="B83" s="43"/>
       <c r="M83" s="2"/>
     </row>
-    <row r="84" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A84" s="39"/>
-      <c r="B84" s="39"/>
+    <row r="84" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A84" s="62"/>
+      <c r="B84" s="42"/>
       <c r="M84" s="2"/>
     </row>
-    <row r="85" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A85" s="57"/>
-      <c r="B85" s="57"/>
+    <row r="85" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A85" s="61"/>
+      <c r="B85" s="43"/>
       <c r="M85" s="2"/>
     </row>
-    <row r="86" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86" s="39"/>
-      <c r="B86" s="39"/>
+    <row r="86" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A86" s="62"/>
+      <c r="B86" s="42"/>
       <c r="M86" s="2"/>
     </row>
-    <row r="87" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A87" s="57"/>
-      <c r="B87" s="57"/>
+    <row r="87" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A87" s="61"/>
+      <c r="B87" s="43"/>
       <c r="M87" s="2"/>
     </row>
-    <row r="88" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A88" s="60"/>
-      <c r="B88" s="61"/>
+    <row r="88" spans="1:13" ht="15" x14ac:dyDescent="0.15">
+      <c r="A88" s="66"/>
+      <c r="B88" s="45"/>
       <c r="C88" s="30"/>
       <c r="M88" s="2"/>
     </row>
-    <row r="89" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A89" s="62"/>
-      <c r="B89" s="63"/>
+    <row r="89" spans="1:13" ht="15" x14ac:dyDescent="0.15">
+      <c r="A89" s="67"/>
+      <c r="B89" s="46"/>
       <c r="C89" s="30"/>
       <c r="M89" s="3"/>
     </row>
-    <row r="90" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A90" s="64"/>
-      <c r="B90" s="61"/>
+    <row r="90" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A90" s="68"/>
+      <c r="B90" s="45"/>
       <c r="C90" s="30"/>
       <c r="M90" s="3"/>
     </row>
-    <row r="91" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A91" s="65"/>
-      <c r="B91" s="63"/>
+    <row r="91" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A91" s="69"/>
+      <c r="B91" s="46"/>
       <c r="C91" s="30"/>
     </row>
-    <row r="92" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A92" s="64"/>
-      <c r="B92" s="61"/>
+    <row r="92" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A92" s="68"/>
+      <c r="B92" s="45"/>
       <c r="C92" s="30"/>
     </row>
-    <row r="93" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A93" s="65"/>
-      <c r="B93" s="63"/>
+    <row r="93" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A93" s="69"/>
+      <c r="B93" s="46"/>
       <c r="C93" s="30"/>
     </row>
-    <row r="94" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A94" s="64"/>
-      <c r="B94" s="61"/>
+    <row r="94" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A94" s="68"/>
+      <c r="B94" s="45"/>
       <c r="C94" s="30"/>
     </row>
-    <row r="95" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A95" s="65"/>
-      <c r="B95" s="63"/>
+    <row r="95" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A95" s="69"/>
+      <c r="B95" s="46"/>
       <c r="C95" s="30"/>
       <c r="H95" s="4"/>
     </row>
-    <row r="96" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A96" s="64"/>
-      <c r="B96" s="61"/>
+    <row r="96" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+      <c r="A96" s="68"/>
+      <c r="B96" s="45"/>
       <c r="C96" s="30"/>
       <c r="H96" s="4"/>
     </row>
-    <row r="97" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A97" s="65"/>
-      <c r="B97" s="63"/>
+    <row r="97" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A97" s="69"/>
+      <c r="B97" s="46"/>
       <c r="C97" s="30"/>
       <c r="G97" s="5"/>
       <c r="H97" s="6"/>
       <c r="I97" s="5"/>
       <c r="J97" s="5"/>
     </row>
-    <row r="98" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A98" s="39"/>
-      <c r="B98" s="39"/>
+    <row r="98" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A98" s="62"/>
+      <c r="B98" s="42"/>
       <c r="G98" s="5"/>
       <c r="H98" s="6"/>
       <c r="I98" s="5"/>
       <c r="J98" s="5"/>
     </row>
-    <row r="99" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A99" s="56"/>
-      <c r="B99" s="63"/>
+    <row r="99" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A99" s="70"/>
+      <c r="B99" s="46"/>
       <c r="C99" s="35"/>
       <c r="G99" s="10"/>
       <c r="H99" s="8"/>
       <c r="I99" s="5"/>
       <c r="J99" s="5"/>
     </row>
-    <row r="100" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A100" s="66"/>
-      <c r="B100" s="61"/>
+    <row r="100" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A100" s="71"/>
+      <c r="B100" s="45"/>
       <c r="C100" s="35"/>
       <c r="G100" s="7"/>
       <c r="H100" s="8"/>
       <c r="I100" s="5"/>
       <c r="J100" s="5"/>
     </row>
-    <row r="101" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A101" s="57"/>
-      <c r="B101" s="63"/>
+    <row r="101" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A101" s="61"/>
+      <c r="B101" s="46"/>
       <c r="C101" s="35"/>
       <c r="G101" s="7"/>
       <c r="H101" s="8"/>
       <c r="I101" s="5"/>
       <c r="J101" s="5"/>
     </row>
-    <row r="102" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A102" s="39"/>
-      <c r="B102" s="61"/>
+    <row r="102" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A102" s="62"/>
+      <c r="B102" s="45"/>
       <c r="C102" s="35"/>
       <c r="G102" s="7"/>
       <c r="H102" s="8"/>
       <c r="I102" s="5"/>
       <c r="J102" s="5"/>
     </row>
-    <row r="103" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A103" s="57"/>
-      <c r="B103" s="63"/>
+    <row r="103" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A103" s="61"/>
+      <c r="B103" s="46"/>
       <c r="C103" s="35"/>
       <c r="G103" s="7"/>
       <c r="H103" s="8"/>
       <c r="I103" s="5"/>
       <c r="J103" s="5"/>
     </row>
-    <row r="104" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A104" s="39"/>
-      <c r="B104" s="61"/>
+    <row r="104" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A104" s="62"/>
+      <c r="B104" s="45"/>
       <c r="C104" s="35"/>
       <c r="G104" s="5"/>
       <c r="H104" s="8"/>
       <c r="I104" s="5"/>
       <c r="J104" s="5"/>
     </row>
-    <row r="105" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A105" s="57"/>
-      <c r="B105" s="63"/>
+    <row r="105" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A105" s="61"/>
+      <c r="B105" s="46"/>
       <c r="C105" s="35"/>
       <c r="G105" s="5"/>
       <c r="H105" s="8"/>
       <c r="I105" s="5"/>
       <c r="J105" s="5"/>
     </row>
-    <row r="106" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A106" s="39"/>
-      <c r="B106" s="61"/>
+    <row r="106" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A106" s="62"/>
+      <c r="B106" s="45"/>
       <c r="C106" s="35"/>
       <c r="G106" s="5"/>
       <c r="H106" s="8"/>
       <c r="I106" s="5"/>
       <c r="J106" s="5"/>
     </row>
-    <row r="107" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A107" s="57"/>
-      <c r="B107" s="63"/>
+    <row r="107" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A107" s="61"/>
+      <c r="B107" s="46"/>
       <c r="C107" s="35"/>
       <c r="G107" s="5"/>
       <c r="H107" s="8"/>
       <c r="I107" s="5"/>
       <c r="J107" s="5"/>
     </row>
-    <row r="108" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A108" s="39"/>
-      <c r="B108" s="61"/>
+    <row r="108" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A108" s="62"/>
+      <c r="B108" s="45"/>
       <c r="C108" s="35"/>
       <c r="G108" s="5"/>
       <c r="H108" s="8"/>
       <c r="I108" s="5"/>
       <c r="J108" s="5"/>
     </row>
-    <row r="109" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A109" s="57"/>
-      <c r="B109" s="57"/>
+    <row r="109" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="72"/>
+      <c r="B109" s="47"/>
       <c r="G109" s="5"/>
       <c r="H109" s="8"/>
       <c r="I109" s="5"/>
       <c r="J109" s="5"/>
     </row>
-    <row r="110" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A110" s="39"/>
-      <c r="B110" s="39"/>
+    <row r="110" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A110" s="37"/>
+      <c r="B110" s="37"/>
       <c r="G110" s="5"/>
       <c r="H110" s="8"/>
       <c r="I110" s="5"/>
       <c r="J110" s="5"/>
     </row>
-    <row r="111" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G111" s="5"/>
       <c r="H111" s="8"/>
       <c r="I111" s="5"/>
       <c r="J111" s="5"/>
     </row>
-    <row r="112" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G112" s="5"/>
       <c r="H112" s="8"/>
       <c r="I112" s="5"/>
       <c r="J112" s="5"/>
     </row>
-    <row r="113" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G113" s="5"/>
       <c r="H113" s="8"/>
       <c r="I113" s="5"/>
       <c r="J113" s="5"/>
     </row>
-    <row r="114" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G114" s="5"/>
       <c r="H114" s="8"/>
       <c r="I114" s="5"/>
       <c r="J114" s="5"/>
     </row>
-    <row r="115" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G115" s="10"/>
       <c r="H115" s="8"/>
       <c r="I115" s="5"/>
       <c r="J115" s="5"/>
     </row>
-    <row r="116" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G116" s="10"/>
       <c r="H116" s="8"/>
       <c r="I116" s="5"/>
       <c r="J116" s="5"/>
     </row>
-    <row r="117" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G117" s="10"/>
       <c r="H117" s="8"/>
       <c r="I117" s="5"/>
       <c r="J117" s="5"/>
     </row>
-    <row r="118" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G118" s="10"/>
       <c r="H118" s="8"/>
       <c r="I118" s="5"/>
       <c r="J118" s="5"/>
     </row>
-    <row r="119" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G119" s="10"/>
       <c r="H119" s="8"/>
       <c r="I119" s="5"/>
       <c r="J119" s="5"/>
     </row>
-    <row r="120" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G120" s="10"/>
       <c r="H120" s="8"/>
       <c r="I120" s="5"/>
       <c r="J120" s="5"/>
     </row>
-    <row r="121" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G121" s="10"/>
       <c r="H121" s="8"/>
       <c r="I121" s="5"/>
       <c r="J121" s="5"/>
     </row>
-    <row r="122" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G122" s="10"/>
       <c r="H122" s="8"/>
       <c r="I122" s="5"/>
       <c r="J122" s="5"/>
     </row>
-    <row r="123" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G123" s="7"/>
       <c r="H123" s="8"/>
       <c r="I123" s="5"/>
       <c r="J123" s="5"/>
     </row>
-    <row r="124" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G124" s="7"/>
       <c r="H124" s="8"/>
       <c r="I124" s="5"/>
       <c r="J124" s="5"/>
     </row>
-    <row r="125" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G125" s="7"/>
       <c r="H125" s="8"/>
       <c r="I125" s="5"/>
       <c r="J125" s="5"/>
     </row>
-    <row r="126" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="126" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G126" s="7"/>
       <c r="H126" s="8"/>
       <c r="I126" s="5"/>
       <c r="J126" s="5"/>
     </row>
-    <row r="127" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G127" s="7"/>
       <c r="H127" s="8"/>
       <c r="I127" s="5"/>
       <c r="J127" s="5"/>
     </row>
-    <row r="128" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="128" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G128" s="7"/>
       <c r="H128" s="8"/>
       <c r="I128" s="5"/>
       <c r="J128" s="5"/>
     </row>
-    <row r="129" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="129" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G129" s="5"/>
       <c r="H129" s="8"/>
       <c r="I129" s="5"/>
       <c r="J129" s="5"/>
     </row>
-    <row r="130" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="130" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G130" s="5"/>
       <c r="H130" s="8"/>
       <c r="I130" s="5"/>
       <c r="J130" s="5"/>
     </row>
-    <row r="131" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="131" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G131" s="5"/>
       <c r="H131" s="9"/>
       <c r="I131" s="5"/>
       <c r="J131" s="5"/>
     </row>
-    <row r="132" spans="7:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="132" spans="7:10" ht="16" x14ac:dyDescent="0.2">
       <c r="G132" s="5"/>
       <c r="H132" s="9"/>
       <c r="I132" s="5"/>
       <c r="J132" s="5"/>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A179" s="11"/>
       <c r="B179" s="12"/>
       <c r="C179" s="12"/>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A180" s="11"/>
       <c r="B180" s="12"/>
       <c r="C180" s="12"/>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A181" s="11"/>
       <c r="B181" s="12"/>
       <c r="C181" s="12"/>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A182" s="11"/>
       <c r="B182" s="12"/>
       <c r="C182" s="12"/>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A183" s="11"/>
       <c r="B183" s="12"/>
       <c r="C183" s="12"/>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A184" s="11"/>
       <c r="B184" s="12"/>
       <c r="C184" s="12"/>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A185" s="11"/>
       <c r="B185" s="12"/>
       <c r="C185" s="12"/>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A186" s="11"/>
       <c r="B186" s="12"/>
       <c r="C186" s="12"/>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A187" s="11"/>
       <c r="B187" s="12"/>
       <c r="C187" s="12"/>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A188" s="11"/>
       <c r="B188" s="12"/>
       <c r="C188" s="12"/>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A189" s="11"/>
       <c r="B189" s="12"/>
       <c r="C189" s="12"/>
     </row>
-    <row r="190" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:3" ht="15" x14ac:dyDescent="0.15">
       <c r="A190" s="11"/>
       <c r="B190" s="13"/>
       <c r="C190" s="12"/>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A191" s="11"/>
       <c r="B191" s="12"/>
       <c r="C191" s="12"/>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A192" s="14"/>
       <c r="B192" s="14"/>
       <c r="C192" s="14"/>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A193" s="15"/>
       <c r="B193" s="16"/>
       <c r="C193" s="16"/>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A194" s="15"/>
       <c r="B194" s="12"/>
       <c r="C194" s="12"/>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A195" s="15"/>
       <c r="B195" s="17"/>
       <c r="C195" s="17"/>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A196" s="14"/>
       <c r="B196" s="18"/>
       <c r="C196" s="18"/>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A197" s="14"/>
       <c r="B197" s="19"/>
       <c r="C197" s="19"/>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A198" s="15"/>
       <c r="B198" s="19"/>
       <c r="C198" s="19"/>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A199" s="20"/>
       <c r="B199" s="12"/>
       <c r="C199" s="12"/>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A200" s="20"/>
       <c r="B200" s="21"/>
       <c r="C200" s="22"/>
       <c r="D200" s="12"/>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A201" s="20"/>
       <c r="B201" s="12"/>
       <c r="C201" s="22"/>
       <c r="D201" s="12"/>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A202" s="15"/>
       <c r="B202" s="23"/>
       <c r="C202" s="12"/>
       <c r="D202" s="12"/>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A203" s="15"/>
       <c r="B203" s="24"/>
       <c r="C203" s="12"/>
       <c r="D203" s="12"/>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A204" s="15"/>
       <c r="B204" s="23"/>
       <c r="C204" s="25"/>
       <c r="D204" s="12"/>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A205" s="14"/>
       <c r="B205" s="12"/>
       <c r="C205" s="26"/>
       <c r="D205" s="12"/>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A206" s="27"/>
       <c r="B206" s="27"/>
       <c r="C206" s="27"/>
       <c r="D206" s="14"/>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D207" s="12"/>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D208" s="12"/>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D209" s="12"/>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D210" s="12"/>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D211" s="12"/>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D212" s="12"/>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D213" s="12"/>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D214" s="12"/>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D215" s="12"/>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D216" s="12"/>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A217" s="28"/>
       <c r="B217" s="29"/>
       <c r="C217" s="30"/>
       <c r="D217" s="12"/>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A218" s="14"/>
       <c r="B218" s="14"/>
       <c r="C218" s="14"/>
       <c r="D218" s="14"/>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D219" s="12"/>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D220" s="12"/>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D221" s="12"/>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D222" s="12"/>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D223" s="12"/>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.15">
       <c r="D224" s="12"/>
     </row>
-    <row r="225" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="225" spans="4:4" x14ac:dyDescent="0.15">
       <c r="D225" s="12"/>
     </row>
-    <row r="226" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="226" spans="4:4" x14ac:dyDescent="0.15">
       <c r="D226" s="12"/>
     </row>
-    <row r="227" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="227" spans="4:4" x14ac:dyDescent="0.15">
       <c r="D227" s="12"/>
     </row>
-    <row r="228" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="228" spans="4:4" x14ac:dyDescent="0.15">
       <c r="D228" s="12"/>
     </row>
-    <row r="229" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="229" spans="4:4" x14ac:dyDescent="0.15">
       <c r="D229" s="12"/>
     </row>
-    <row r="230" spans="4:4" x14ac:dyDescent="0.2">
+    <row r="230" spans="4:4" x14ac:dyDescent="0.15">
       <c r="D230" s="12"/>
     </row>
   </sheetData>
@@ -2319,6 +2729,22 @@
     <mergeCell ref="A61:B61"/>
     <mergeCell ref="A81:B81"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B41 B43:B60 B62:B80 B82:B109">
+    <cfRule type="expression" dxfId="7" priority="3">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="4">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:A41 A43:A60 A62:A80 A82:A109">
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="1" stopIfTrue="1">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations disablePrompts="1" count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C202:C203" xr:uid="{965493E7-47D2-524D-97B0-AC90AE968230}">
       <formula1>$N$11:$N$61</formula1>

</xml_diff>

<commit_message>
major gui refactoring/additions, corrections to update script, continued integration of report templates
</commit_message>
<xml_diff>
--- a/EconAutomation/src/supporting_docs/econ_wb_templates/Case_Variables.xlsx
+++ b/EconAutomation/src/supporting_docs/econ_wb_templates/Case_Variables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmacbook/Documents/GitHub/EconAutomation-REP/EconAutomation/src/supporting_docs/econ_wb_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88BB1DF8-7904-9646-A5B6-0A4CFFB99F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DC48993-C62F-0F4D-9ABD-E23B029671DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="720" windowWidth="32000" windowHeight="20080" xr2:uid="{765FF91D-C91B-E74A-AE6E-CE36BB29D05E}"/>
   </bookViews>
@@ -665,7 +665,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -766,16 +766,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -788,30 +787,17 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -847,11 +833,20 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -862,47 +857,7 @@
     <cellStyle name="Normal 2" xfId="2" xr:uid="{6F2027E1-5DA8-B64C-9928-C7D64A51A230}"/>
     <cellStyle name="Percent 2" xfId="4" xr:uid="{F9E35F16-9AB0-2F47-9A1E-E8B3AF0707E3}"/>
   </cellStyles>
-  <dxfs count="16">
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <font>
         <color theme="1"/>
@@ -991,254 +946,6 @@
         </right>
         <top/>
         <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right style="thin">
-          <color theme="0"/>
-        </right>
-        <top style="thin">
-          <color theme="0"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right style="thin">
-          <color theme="0"/>
-        </right>
-        <top style="thin">
-          <color theme="0"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right style="thin">
-          <color theme="0"/>
-        </right>
-        <top style="thin">
-          <color theme="0"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="0"/>
-        </left>
-        <right style="thin">
-          <color theme="0"/>
-        </right>
-        <top style="thin">
-          <color theme="0"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-4.9989318521683403E-2"/>
-        </bottom>
         <vertical/>
         <horizontal/>
       </border>
@@ -1591,203 +1298,203 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25" x14ac:dyDescent="0.15">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="66" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="55"/>
+      <c r="B1" s="66"/>
       <c r="C1" s="36"/>
     </row>
     <row r="2" spans="1:3" ht="20" x14ac:dyDescent="0.15">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="54"/>
+      <c r="B2" s="67"/>
       <c r="C2" s="31"/>
     </row>
     <row r="3" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="53"/>
+      <c r="B3" s="50"/>
       <c r="C3" s="32"/>
     </row>
     <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="52" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="38"/>
       <c r="C4" s="22"/>
     </row>
     <row r="5" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="52" t="s">
         <v>32</v>
       </c>
       <c r="B5" s="38"/>
       <c r="C5" s="22"/>
     </row>
     <row r="6" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="52" t="s">
         <v>27</v>
       </c>
       <c r="B6" s="38"/>
       <c r="C6" s="22"/>
     </row>
     <row r="7" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="52" t="s">
         <v>33</v>
       </c>
       <c r="B7" s="38"/>
       <c r="C7" s="12"/>
     </row>
     <row r="8" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A8" s="58" t="s">
+      <c r="A8" s="52" t="s">
         <v>34</v>
       </c>
       <c r="B8" s="38"/>
       <c r="C8" s="12"/>
     </row>
     <row r="9" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A9" s="58" t="s">
+      <c r="A9" s="52" t="s">
         <v>28</v>
       </c>
       <c r="B9" s="38"/>
       <c r="C9" s="12"/>
     </row>
     <row r="10" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="52" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="38"/>
       <c r="C10" s="17"/>
     </row>
     <row r="11" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A11" s="58" t="s">
+      <c r="A11" s="52" t="s">
         <v>6</v>
       </c>
       <c r="B11" s="38"/>
       <c r="C11" s="17"/>
     </row>
     <row r="12" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A12" s="58" t="s">
+      <c r="A12" s="52" t="s">
         <v>2</v>
       </c>
       <c r="B12" s="38"/>
       <c r="C12" s="17"/>
     </row>
     <row r="13" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A13" s="58" t="s">
+      <c r="A13" s="52" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="38"/>
       <c r="C13" s="17"/>
     </row>
     <row r="14" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A14" s="58" t="s">
+      <c r="A14" s="52" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="38"/>
       <c r="C14" s="17"/>
     </row>
     <row r="15" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A15" s="58" t="s">
+      <c r="A15" s="52" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="39"/>
       <c r="C15" s="17"/>
     </row>
     <row r="16" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A16" s="58" t="s">
+      <c r="A16" s="52" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="39"/>
       <c r="C16" s="17"/>
     </row>
     <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A17" s="58" t="s">
+      <c r="A17" s="52" t="s">
         <v>3</v>
       </c>
       <c r="B17" s="39"/>
       <c r="C17" s="17"/>
     </row>
     <row r="18" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A18" s="58" t="s">
+      <c r="A18" s="52" t="s">
         <v>35</v>
       </c>
       <c r="B18" s="39"/>
       <c r="C18" s="17"/>
     </row>
     <row r="19" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A19" s="58" t="s">
+      <c r="A19" s="52" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="39"/>
       <c r="C19" s="17"/>
     </row>
     <row r="20" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A20" s="58" t="s">
+      <c r="A20" s="52" t="s">
         <v>21</v>
       </c>
       <c r="B20" s="39"/>
       <c r="C20" s="17"/>
     </row>
     <row r="21" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A21" s="58" t="s">
+      <c r="A21" s="52" t="s">
         <v>36</v>
       </c>
       <c r="B21" s="38"/>
       <c r="C21" s="26"/>
     </row>
     <row r="22" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A22" s="58" t="s">
+      <c r="A22" s="52" t="s">
         <v>22</v>
       </c>
       <c r="B22" s="38"/>
       <c r="C22" s="26"/>
     </row>
     <row r="23" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A23" s="58" t="s">
+      <c r="A23" s="52" t="s">
         <v>23</v>
       </c>
       <c r="B23" s="39"/>
       <c r="C23" s="26"/>
     </row>
     <row r="24" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A24" s="58" t="s">
+      <c r="A24" s="52" t="s">
         <v>37</v>
       </c>
       <c r="B24" s="39"/>
       <c r="C24" s="26"/>
     </row>
     <row r="25" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A25" s="58" t="s">
+      <c r="A25" s="52" t="s">
         <v>24</v>
       </c>
       <c r="B25" s="39"/>
       <c r="C25" s="26"/>
     </row>
     <row r="26" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A26" s="58" t="s">
+      <c r="A26" s="52" t="s">
         <v>25</v>
       </c>
       <c r="B26" s="39"/>
       <c r="C26" s="26"/>
     </row>
     <row r="27" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A27" s="58" t="s">
+      <c r="A27" s="52" t="s">
         <v>55</v>
       </c>
       <c r="B27" s="39"/>
       <c r="C27" s="26"/>
     </row>
     <row r="28" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A28" s="58" t="s">
+      <c r="A28" s="52" t="s">
         <v>56</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A29" s="58" t="s">
+      <c r="A29" s="52" t="s">
         <v>29</v>
       </c>
       <c r="B29" s="39"/>
@@ -1796,7 +1503,7 @@
       </c>
     </row>
     <row r="30" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A30" s="58" t="s">
+      <c r="A30" s="52" t="s">
         <v>30</v>
       </c>
       <c r="B30" s="39"/>
@@ -1805,7 +1512,7 @@
       </c>
     </row>
     <row r="31" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A31" s="58" t="s">
+      <c r="A31" s="52" t="s">
         <v>31</v>
       </c>
       <c r="B31" s="39"/>
@@ -1814,7 +1521,7 @@
       </c>
     </row>
     <row r="32" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A32" s="58" t="s">
+      <c r="A32" s="52" t="s">
         <v>0</v>
       </c>
       <c r="B32" s="39"/>
@@ -1823,7 +1530,7 @@
       </c>
     </row>
     <row r="33" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A33" s="58" t="s">
+      <c r="A33" s="52" t="s">
         <v>58</v>
       </c>
       <c r="B33" s="39"/>
@@ -1832,7 +1539,7 @@
       </c>
     </row>
     <row r="34" spans="1:3" ht="15" x14ac:dyDescent="0.15">
-      <c r="A34" s="58" t="s">
+      <c r="A34" s="52" t="s">
         <v>59</v>
       </c>
       <c r="B34" s="40"/>
@@ -1841,7 +1548,7 @@
       </c>
     </row>
     <row r="35" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A35" s="58" t="s">
+      <c r="A35" s="52" t="s">
         <v>60</v>
       </c>
       <c r="B35" s="41"/>
@@ -1850,7 +1557,7 @@
       </c>
     </row>
     <row r="36" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A36" s="58" t="s">
+      <c r="A36" s="52" t="s">
         <v>68</v>
       </c>
       <c r="B36" s="41"/>
@@ -1859,7 +1566,7 @@
       </c>
     </row>
     <row r="37" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A37" s="58" t="s">
+      <c r="A37" s="52" t="s">
         <v>69</v>
       </c>
       <c r="B37" s="41"/>
@@ -1868,7 +1575,7 @@
       </c>
     </row>
     <row r="38" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A38" s="58" t="s">
+      <c r="A38" s="52" t="s">
         <v>70</v>
       </c>
       <c r="B38" s="41"/>
@@ -1877,7 +1584,7 @@
       </c>
     </row>
     <row r="39" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A39" s="58" t="s">
+      <c r="A39" s="52" t="s">
         <v>71</v>
       </c>
       <c r="B39" s="41"/>
@@ -1886,364 +1593,364 @@
       </c>
     </row>
     <row r="40" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A40" s="58"/>
+      <c r="A40" s="52"/>
       <c r="B40" s="41"/>
       <c r="C40" s="14"/>
     </row>
     <row r="41" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A41" s="59"/>
-      <c r="B41" s="51"/>
+      <c r="A41" s="53"/>
+      <c r="B41" s="49"/>
       <c r="C41" s="14"/>
     </row>
     <row r="42" spans="1:3" ht="20" x14ac:dyDescent="0.15">
-      <c r="A42" s="52" t="s">
+      <c r="A42" s="68" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="52"/>
+      <c r="B42" s="68"/>
       <c r="C42" s="33"/>
     </row>
     <row r="43" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A43" s="60" t="s">
+      <c r="A43" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="B43" s="49"/>
+      <c r="B43" s="48"/>
     </row>
     <row r="44" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A44" s="61" t="s">
+      <c r="A44" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="B44" s="43"/>
+      <c r="B44" s="42"/>
     </row>
     <row r="45" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A45" s="62" t="s">
+      <c r="A45" s="56" t="s">
         <v>39</v>
       </c>
-      <c r="B45" s="42"/>
+      <c r="B45" s="41"/>
     </row>
     <row r="46" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A46" s="61" t="s">
+      <c r="A46" s="55" t="s">
         <v>74</v>
       </c>
-      <c r="B46" s="43"/>
+      <c r="B46" s="42"/>
     </row>
     <row r="47" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A47" s="63" t="s">
+      <c r="A47" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="B47" s="44"/>
+      <c r="B47" s="43"/>
     </row>
     <row r="48" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A48" s="61" t="s">
+      <c r="A48" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="B48" s="43"/>
+      <c r="B48" s="42"/>
     </row>
     <row r="49" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A49" s="63" t="s">
+      <c r="A49" s="57" t="s">
         <v>75</v>
       </c>
-      <c r="B49" s="44"/>
+      <c r="B49" s="43"/>
     </row>
     <row r="50" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A50" s="61" t="s">
+      <c r="A50" s="55" t="s">
         <v>76</v>
       </c>
-      <c r="B50" s="43"/>
+      <c r="B50" s="42"/>
     </row>
     <row r="51" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A51" s="63" t="s">
+      <c r="A51" s="57" t="s">
         <v>61</v>
       </c>
-      <c r="B51" s="44"/>
+      <c r="B51" s="43"/>
       <c r="C51" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A52" s="61" t="s">
+      <c r="A52" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="B52" s="43"/>
+      <c r="B52" s="42"/>
       <c r="C52" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A53" s="63" t="s">
+      <c r="A53" s="57" t="s">
         <v>63</v>
       </c>
-      <c r="B53" s="44"/>
+      <c r="B53" s="43"/>
       <c r="C53" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A54" s="61" t="s">
+      <c r="A54" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="B54" s="43"/>
+      <c r="B54" s="42"/>
       <c r="C54" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A55" s="63" t="s">
+      <c r="A55" s="57" t="s">
         <v>65</v>
       </c>
-      <c r="B55" s="44"/>
+      <c r="B55" s="43"/>
       <c r="C55" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A56" s="61" t="s">
+      <c r="A56" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="B56" s="43"/>
+      <c r="B56" s="42"/>
     </row>
     <row r="57" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A57" s="63" t="s">
+      <c r="A57" s="57" t="s">
         <v>42</v>
       </c>
-      <c r="B57" s="44"/>
+      <c r="B57" s="43"/>
     </row>
     <row r="58" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A58" s="61" t="s">
+      <c r="A58" s="55" t="s">
         <v>43</v>
       </c>
-      <c r="B58" s="43"/>
+      <c r="B58" s="42"/>
     </row>
     <row r="59" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A59" s="63" t="s">
+      <c r="A59" s="57" t="s">
         <v>44</v>
       </c>
-      <c r="B59" s="44"/>
+      <c r="B59" s="43"/>
     </row>
     <row r="60" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A60" s="64"/>
-      <c r="B60" s="48"/>
+      <c r="A60" s="58"/>
+      <c r="B60" s="47"/>
     </row>
     <row r="61" spans="1:3" ht="20" x14ac:dyDescent="0.25">
-      <c r="A61" s="50" t="s">
+      <c r="A61" s="69" t="s">
         <v>67</v>
       </c>
-      <c r="B61" s="50"/>
+      <c r="B61" s="69"/>
       <c r="C61" s="34"/>
     </row>
     <row r="62" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A62" s="60" t="s">
+      <c r="A62" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="B62" s="49"/>
+      <c r="B62" s="48"/>
     </row>
     <row r="63" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A63" s="61" t="s">
+      <c r="A63" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="B63" s="43"/>
+      <c r="B63" s="42"/>
     </row>
     <row r="64" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A64" s="62" t="s">
+      <c r="A64" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="B64" s="42"/>
+      <c r="B64" s="41"/>
     </row>
     <row r="65" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A65" s="61" t="s">
+      <c r="A65" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="B65" s="43"/>
+      <c r="B65" s="42"/>
     </row>
     <row r="66" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A66" s="62" t="s">
+      <c r="A66" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="B66" s="42"/>
+      <c r="B66" s="41"/>
     </row>
     <row r="67" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A67" s="61" t="s">
+      <c r="A67" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="B67" s="43"/>
+      <c r="B67" s="42"/>
     </row>
     <row r="68" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A68" s="62" t="s">
+      <c r="A68" s="56" t="s">
         <v>47</v>
       </c>
-      <c r="B68" s="42"/>
+      <c r="B68" s="41"/>
     </row>
     <row r="69" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A69" s="61" t="s">
+      <c r="A69" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="B69" s="43"/>
+      <c r="B69" s="42"/>
     </row>
     <row r="70" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A70" s="62" t="s">
+      <c r="A70" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="B70" s="42"/>
+      <c r="B70" s="41"/>
       <c r="M70" s="2"/>
     </row>
     <row r="71" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A71" s="61" t="s">
+      <c r="A71" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="B71" s="43"/>
+      <c r="B71" s="42"/>
       <c r="M71" s="2"/>
     </row>
     <row r="72" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A72" s="62" t="s">
+      <c r="A72" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="B72" s="42"/>
+      <c r="B72" s="41"/>
       <c r="M72" s="2"/>
     </row>
     <row r="73" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A73" s="61" t="s">
+      <c r="A73" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="B73" s="43"/>
+      <c r="B73" s="42"/>
       <c r="M73" s="2"/>
     </row>
     <row r="74" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A74" s="62" t="s">
+      <c r="A74" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="B74" s="42"/>
+      <c r="B74" s="41"/>
       <c r="M74" s="2"/>
     </row>
     <row r="75" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A75" s="61" t="s">
+      <c r="A75" s="55" t="s">
         <v>50</v>
       </c>
-      <c r="B75" s="43"/>
+      <c r="B75" s="42"/>
       <c r="M75" s="2"/>
     </row>
     <row r="76" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A76" s="62" t="s">
+      <c r="A76" s="56" t="s">
         <v>51</v>
       </c>
-      <c r="B76" s="42"/>
+      <c r="B76" s="41"/>
       <c r="M76" s="2"/>
     </row>
     <row r="77" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A77" s="61" t="s">
+      <c r="A77" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="B77" s="43"/>
+      <c r="B77" s="42"/>
       <c r="M77" s="2"/>
     </row>
     <row r="78" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A78" s="62" t="s">
+      <c r="A78" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="B78" s="42"/>
+      <c r="B78" s="41"/>
       <c r="M78" s="2"/>
     </row>
     <row r="79" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A79" s="61" t="s">
+      <c r="A79" s="55" t="s">
         <v>54</v>
       </c>
-      <c r="B79" s="43"/>
+      <c r="B79" s="42"/>
       <c r="M79" s="2"/>
     </row>
     <row r="80" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A80" s="65"/>
-      <c r="B80" s="56"/>
+      <c r="A80" s="59"/>
+      <c r="B80" s="49"/>
       <c r="M80" s="2"/>
     </row>
     <row r="81" spans="1:13" ht="20" x14ac:dyDescent="0.25">
-      <c r="A81" s="50" t="s">
+      <c r="A81" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="B81" s="50"/>
+      <c r="B81" s="69"/>
       <c r="C81" s="34"/>
       <c r="M81" s="2"/>
     </row>
     <row r="82" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A82" s="60"/>
-      <c r="B82" s="49"/>
+      <c r="A82" s="54"/>
+      <c r="B82" s="48"/>
       <c r="M82" s="2"/>
     </row>
     <row r="83" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A83" s="61"/>
-      <c r="B83" s="43"/>
+      <c r="A83" s="55"/>
+      <c r="B83" s="42"/>
       <c r="M83" s="2"/>
     </row>
     <row r="84" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A84" s="62"/>
-      <c r="B84" s="42"/>
+      <c r="A84" s="56"/>
+      <c r="B84" s="41"/>
       <c r="M84" s="2"/>
     </row>
     <row r="85" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A85" s="61"/>
-      <c r="B85" s="43"/>
+      <c r="A85" s="55"/>
+      <c r="B85" s="42"/>
       <c r="M85" s="2"/>
     </row>
     <row r="86" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A86" s="62"/>
-      <c r="B86" s="42"/>
+      <c r="A86" s="56"/>
+      <c r="B86" s="41"/>
       <c r="M86" s="2"/>
     </row>
     <row r="87" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A87" s="61"/>
-      <c r="B87" s="43"/>
+      <c r="A87" s="55"/>
+      <c r="B87" s="42"/>
       <c r="M87" s="2"/>
     </row>
     <row r="88" spans="1:13" ht="15" x14ac:dyDescent="0.15">
-      <c r="A88" s="66"/>
-      <c r="B88" s="45"/>
+      <c r="A88" s="60"/>
+      <c r="B88" s="44"/>
       <c r="C88" s="30"/>
       <c r="M88" s="2"/>
     </row>
     <row r="89" spans="1:13" ht="15" x14ac:dyDescent="0.15">
-      <c r="A89" s="67"/>
-      <c r="B89" s="46"/>
+      <c r="A89" s="61"/>
+      <c r="B89" s="45"/>
       <c r="C89" s="30"/>
       <c r="M89" s="3"/>
     </row>
     <row r="90" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A90" s="68"/>
-      <c r="B90" s="45"/>
+      <c r="A90" s="62"/>
+      <c r="B90" s="44"/>
       <c r="C90" s="30"/>
       <c r="M90" s="3"/>
     </row>
     <row r="91" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A91" s="69"/>
-      <c r="B91" s="46"/>
+      <c r="A91" s="63"/>
+      <c r="B91" s="45"/>
       <c r="C91" s="30"/>
     </row>
     <row r="92" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A92" s="68"/>
-      <c r="B92" s="45"/>
+      <c r="A92" s="62"/>
+      <c r="B92" s="44"/>
       <c r="C92" s="30"/>
     </row>
     <row r="93" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A93" s="69"/>
-      <c r="B93" s="46"/>
+      <c r="A93" s="63"/>
+      <c r="B93" s="45"/>
       <c r="C93" s="30"/>
     </row>
     <row r="94" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A94" s="68"/>
-      <c r="B94" s="45"/>
+      <c r="A94" s="62"/>
+      <c r="B94" s="44"/>
       <c r="C94" s="30"/>
     </row>
     <row r="95" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A95" s="69"/>
-      <c r="B95" s="46"/>
+      <c r="A95" s="63"/>
+      <c r="B95" s="45"/>
       <c r="C95" s="30"/>
       <c r="H95" s="4"/>
     </row>
     <row r="96" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A96" s="68"/>
-      <c r="B96" s="45"/>
+      <c r="A96" s="62"/>
+      <c r="B96" s="44"/>
       <c r="C96" s="30"/>
       <c r="H96" s="4"/>
     </row>
     <row r="97" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A97" s="69"/>
-      <c r="B97" s="46"/>
+      <c r="A97" s="63"/>
+      <c r="B97" s="45"/>
       <c r="C97" s="30"/>
       <c r="G97" s="5"/>
       <c r="H97" s="6"/>
@@ -2251,16 +1958,16 @@
       <c r="J97" s="5"/>
     </row>
     <row r="98" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A98" s="62"/>
-      <c r="B98" s="42"/>
+      <c r="A98" s="56"/>
+      <c r="B98" s="41"/>
       <c r="G98" s="5"/>
       <c r="H98" s="6"/>
       <c r="I98" s="5"/>
       <c r="J98" s="5"/>
     </row>
     <row r="99" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A99" s="70"/>
-      <c r="B99" s="46"/>
+      <c r="A99" s="64"/>
+      <c r="B99" s="45"/>
       <c r="C99" s="35"/>
       <c r="G99" s="10"/>
       <c r="H99" s="8"/>
@@ -2268,8 +1975,8 @@
       <c r="J99" s="5"/>
     </row>
     <row r="100" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A100" s="71"/>
-      <c r="B100" s="45"/>
+      <c r="A100" s="52"/>
+      <c r="B100" s="44"/>
       <c r="C100" s="35"/>
       <c r="G100" s="7"/>
       <c r="H100" s="8"/>
@@ -2277,8 +1984,8 @@
       <c r="J100" s="5"/>
     </row>
     <row r="101" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A101" s="61"/>
-      <c r="B101" s="46"/>
+      <c r="A101" s="55"/>
+      <c r="B101" s="45"/>
       <c r="C101" s="35"/>
       <c r="G101" s="7"/>
       <c r="H101" s="8"/>
@@ -2286,8 +1993,8 @@
       <c r="J101" s="5"/>
     </row>
     <row r="102" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A102" s="62"/>
-      <c r="B102" s="45"/>
+      <c r="A102" s="56"/>
+      <c r="B102" s="44"/>
       <c r="C102" s="35"/>
       <c r="G102" s="7"/>
       <c r="H102" s="8"/>
@@ -2295,8 +2002,8 @@
       <c r="J102" s="5"/>
     </row>
     <row r="103" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A103" s="61"/>
-      <c r="B103" s="46"/>
+      <c r="A103" s="55"/>
+      <c r="B103" s="45"/>
       <c r="C103" s="35"/>
       <c r="G103" s="7"/>
       <c r="H103" s="8"/>
@@ -2304,8 +2011,8 @@
       <c r="J103" s="5"/>
     </row>
     <row r="104" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A104" s="62"/>
-      <c r="B104" s="45"/>
+      <c r="A104" s="56"/>
+      <c r="B104" s="44"/>
       <c r="C104" s="35"/>
       <c r="G104" s="5"/>
       <c r="H104" s="8"/>
@@ -2313,8 +2020,8 @@
       <c r="J104" s="5"/>
     </row>
     <row r="105" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A105" s="61"/>
-      <c r="B105" s="46"/>
+      <c r="A105" s="55"/>
+      <c r="B105" s="45"/>
       <c r="C105" s="35"/>
       <c r="G105" s="5"/>
       <c r="H105" s="8"/>
@@ -2322,8 +2029,8 @@
       <c r="J105" s="5"/>
     </row>
     <row r="106" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A106" s="62"/>
-      <c r="B106" s="45"/>
+      <c r="A106" s="56"/>
+      <c r="B106" s="44"/>
       <c r="C106" s="35"/>
       <c r="G106" s="5"/>
       <c r="H106" s="8"/>
@@ -2331,8 +2038,8 @@
       <c r="J106" s="5"/>
     </row>
     <row r="107" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A107" s="61"/>
-      <c r="B107" s="46"/>
+      <c r="A107" s="55"/>
+      <c r="B107" s="45"/>
       <c r="C107" s="35"/>
       <c r="G107" s="5"/>
       <c r="H107" s="8"/>
@@ -2340,8 +2047,8 @@
       <c r="J107" s="5"/>
     </row>
     <row r="108" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A108" s="62"/>
-      <c r="B108" s="45"/>
+      <c r="A108" s="56"/>
+      <c r="B108" s="44"/>
       <c r="C108" s="35"/>
       <c r="G108" s="5"/>
       <c r="H108" s="8"/>
@@ -2349,8 +2056,8 @@
       <c r="J108" s="5"/>
     </row>
     <row r="109" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="72"/>
-      <c r="B109" s="47"/>
+      <c r="A109" s="65"/>
+      <c r="B109" s="46"/>
       <c r="G109" s="5"/>
       <c r="H109" s="8"/>
       <c r="I109" s="5"/>
@@ -2729,19 +2436,19 @@
     <mergeCell ref="A61:B61"/>
     <mergeCell ref="A81:B81"/>
   </mergeCells>
-  <conditionalFormatting sqref="B3:B41 B43:B60 B62:B80 B82:B109">
-    <cfRule type="expression" dxfId="7" priority="3">
+  <conditionalFormatting sqref="A3:A41 A43:A60 A62:A80 A82:A109">
+    <cfRule type="expression" dxfId="3" priority="1" stopIfTrue="1">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="4">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3:A41 A43:A60 A62:A80 A82:A109">
-    <cfRule type="expression" dxfId="4" priority="2">
+  <conditionalFormatting sqref="B3:B41 B43:B60 B62:B80 B82:B109">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>ISODD(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="4">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>